<commit_message>
HND arms (SWD/NCC): courses read from the matric number
The arm is part of a class: read from the 4th of the last seven matric
digits (3211... SWD, 3212... NCC) and never chosen. Classes and programme
lengths live in config/classes.php, so a new HND arm or a split ND is a
config change.

- users.arm, nominal_roll.arm and elections.arms, backfilled from matric
  numbers; the matric setter keeps the arm in step
- SchoolClass and Arms helpers: 17 classes by programme length
- the roll is kept per arm: one class select, a Course line in the
  template and the file, and a check of the arm digit
- bulk accounts, the elections form (Courses), eligibility, electorate and
  summary all know the arm
- arms on the profile, home page and admin users (with a filter)
- demo admin and governor now have SWD and NCC matric numbers

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SyKQdpHKCfeE8ibJZk7MaD
</commit_message>
<xml_diff>
--- a/resources/templates/nominal-roll.xlsx
+++ b/resources/templates/nominal-roll.xlsx
@@ -571,7 +571,24 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>{{ARM}}</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>{{ARM_HINT}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>One student per row, from row 6 down. Don't change the green headings.</t>
         </is>
@@ -5600,7 +5617,10 @@
       <formula>AND($A6&lt;&gt;"",COUNTIF($A$6:$A$1005,$A6)&gt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="6">
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Course" error="{{ARM_HINT}}" type="list">
+      <formula1>"{{ARM_LIST}}"</formula1>
+    </dataValidation>
     <dataValidation sqref="B1" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Programme" error="Pick Full-time, Part-time or CODFEL." type="list">
       <formula1>"Full-time,Part-time,CODFEL"</formula1>
     </dataValidation>
@@ -5665,7 +5685,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>At the top of the "Nominal roll" sheet: the programme and level (an admin may have filled these in already). One class per file.</t>
+          <t>At the top of the "Nominal roll" sheet: the programme, level and, for HND, the course (an admin may have filled these in already). One class per file.</t>
         </is>
       </c>
     </row>

</xml_diff>